<commit_message>
get more financial data
</commit_message>
<xml_diff>
--- a/20250812_Finance/01_source/CN FS Hierarchy.xlsx
+++ b/20250812_Finance/01_source/CN FS Hierarchy.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/renjinhu/Desktop/template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\AI_Power_Studio\20250812_Finance\01_source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA51B6D-F91E-B545-A6BB-3B39563402DE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE09AAC-B6CA-4954-B989-280FA08D7257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="1660" windowWidth="22940" windowHeight="12020" activeTab="1" xr2:uid="{27D7EAB7-9D2F-4E6A-9245-2B5EF4B9323F}"/>
+    <workbookView xWindow="6000" yWindow="4110" windowWidth="28800" windowHeight="15370" activeTab="2" xr2:uid="{27D7EAB7-9D2F-4E6A-9245-2B5EF4B9323F}"/>
   </bookViews>
   <sheets>
     <sheet name="BS Hierarchy-Other" sheetId="1" r:id="rId1"/>
     <sheet name="PL Hierarchy-Other" sheetId="2" r:id="rId2"/>
+    <sheet name="metadata" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PL Hierarchy-Other'!$A$1:$C$32</definedName>
@@ -24,31 +25,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="172">
   <si>
     <t>流动资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>非流动资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>固定资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>在建工程</t>
@@ -64,7 +57,7 @@
   </si>
   <si>
     <t>流动负债</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>应付账款</t>
@@ -86,7 +79,7 @@
   </si>
   <si>
     <t>非流动负债</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>租赁负债</t>
@@ -99,27 +92,27 @@
   </si>
   <si>
     <t>资产总计</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>负债合计</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>流动资产合计</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>非流动资产合计</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>流动负债合计</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>非流动负债合计</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>其他应收款</t>
@@ -147,27 +140,27 @@
   </si>
   <si>
     <t xml:space="preserve">   主营业务收入</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">   其他业务收入</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">   主营业务成本</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">   其他业务成本</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>毛利</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>毛利率</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>税金及附加</t>
@@ -192,129 +185,129 @@
   </si>
   <si>
     <t xml:space="preserve">           其中：利息费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>营业外收入</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>营业外支出</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>所得税费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>营业利润/(亏损)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>税前利润/(亏损)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>净利润/(亏损)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>资产减值损益</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>公允价值变动损益</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>信用减值损益</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>补贴收入</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>投资收益</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>负债及所有者权益</t>
   </si>
   <si>
     <t>资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>流动资产</t>
   </si>
   <si>
     <t xml:space="preserve">       货币资金</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       交易性金融资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       其他应收款</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       预付款项</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       存货</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       长期股权投资</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">               固定资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">               累计折旧</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       固定资产-净值</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       在建工程</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       无形资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       商誉</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       使用权资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       长期待摊费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       其他非流动资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       其他流动资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>固定资产-净值</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>商誉</t>
@@ -330,23 +323,23 @@
   </si>
   <si>
     <t>使用权资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>报表项目</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>报表项目显示</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>资  产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>负  债  及  所  有  者  权  益</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>非流动负债</t>
@@ -365,117 +358,117 @@
   </si>
   <si>
     <t xml:space="preserve">       应付账款</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       实收资本</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>所有者权益</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       租赁负债</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       预计负债</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       递延收益</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       长期应付职工薪酬</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       其他非流动负债</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       递延所得税负债</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       资本公积</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       衍生金融负债</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       合同负债</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       应付职工薪酬</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       应交税费</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       其他应付款</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       一年内到期的非流动负债</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       其他流动负债</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       盈余公积</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       未分配利润</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">  归属于母公司所有者权益合计</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">  少数股东权益</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>递延所得税资产</t>
   </si>
   <si>
     <t xml:space="preserve">       递延所得税资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       应收账款</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>应收账款</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       应收票据</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>所有者权益</t>
   </si>
   <si>
     <t>主营业务收入</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>其他业务收入</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>补贴收入</t>
@@ -500,35 +493,35 @@
   </si>
   <si>
     <t>主营业务成本</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>其他业务成本</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>其中：利息费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>利息收入</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>所有者权益合计</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>负债及所有者权益总计</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>营业收入</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>财务费用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>营业利润/(亏损)</t>
@@ -541,84 +534,156 @@
   </si>
   <si>
     <t>营业成本</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>实收资本</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>应收票据</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>交易性金融资产</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>长期股权投资</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>预付款项</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>累计折旧</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>应付职工薪酬</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       应付股利</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>应付股利</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>货币资金</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>应收款项融资</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">       应收款项融资</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">  其他综合收益</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>其他综合收益</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>No.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>No.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Account</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>FA</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mgmt GAAP Account</t>
+  </si>
+  <si>
+    <t>Mgmt GAAP Description</t>
+  </si>
+  <si>
+    <t>Local GAAP Account</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Local GAAP Description - English</t>
+  </si>
+  <si>
+    <t>Local GAAP Description - Chinese</t>
+  </si>
+  <si>
+    <t>BS/PL</t>
+  </si>
+  <si>
+    <t>Fixed TB</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Roll forward</t>
+  </si>
+  <si>
+    <t>Adjustment</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>PRC Final TB</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mgmt GAAP Description</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mgmt GAAP Account</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>Local GAAP Account</t>
+  </si>
+  <si>
+    <t>Fixed TB</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>BS/PL</t>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="#,##0;[Red]\-#,##0;&quot;－&quot;"/>
+  </numFmts>
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
       <family val="2"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -677,6 +742,25 @@
       <family val="4"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="ＭＳ ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="4">
@@ -739,68 +823,536 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="177" fontId="11" fillId="0" borderId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="4">
+    <cellStyle name="Comma" xfId="1" xr:uid="{097FE902-4282-40CD-950E-5346F88D78D1}"/>
+    <cellStyle name="Comma 4 2" xfId="2" xr:uid="{D2CEF5E6-3C55-4E50-AD9E-E823DFD9553B}"/>
+    <cellStyle name="標準 3" xfId="3" xr:uid="{1979D52C-7D27-4199-9A28-15FBE535E17A}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="37">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9C0006"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9C0006"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9C0006"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9C0006"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -823,16 +1375,6 @@
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -850,8 +1392,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3FE30168-B15B-4C7B-B45E-57CE7E55A121}" name="Table1" displayName="Table1" ref="A1:C65" totalsRowShown="0">
   <autoFilter ref="A1:C65" xr:uid="{3FE30168-B15B-4C7B-B45E-57CE7E55A121}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{7D4FF766-89C6-4BA3-8D9A-3D5F5ED329D5}" name="No." dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{D45F91AA-BFDE-4A7E-964A-15EA57A2A891}" name="报表项目显示" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{7D4FF766-89C6-4BA3-8D9A-3D5F5ED329D5}" name="No." dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{D45F91AA-BFDE-4A7E-964A-15EA57A2A891}" name="报表项目显示" dataDxfId="35"/>
     <tableColumn id="3" xr3:uid="{5C378BA8-D428-4C5E-9676-6C4A2CE181E9}" name="报表项目"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1176,7 +1718,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FFD7424-6E04-4A31-8F24-5E15AE74A08B}">
   <dimension ref="A1:C65"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="10" style="4" customWidth="1"/>
     <col min="2" max="2" width="33.83203125" customWidth="1"/>
@@ -1294,13 +1836,13 @@
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="10">
+      <c r="A11" s="4">
         <v>10</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" t="s">
         <v>149</v>
       </c>
     </row>
@@ -1362,7 +1904,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="16" outlineLevel="1">
+    <row r="18" spans="1:3" outlineLevel="1">
       <c r="A18" s="4">
         <v>16</v>
       </c>
@@ -1589,10 +2131,10 @@
       <c r="A40" s="4">
         <v>36</v>
       </c>
-      <c r="B40" s="13" t="s">
+      <c r="B40" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="C40" s="12" t="s">
+      <c r="C40" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1804,10 +2346,10 @@
       <c r="A62" s="4">
         <v>55</v>
       </c>
-      <c r="B62" s="13" t="s">
+      <c r="B62" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="C62" s="12" t="s">
+      <c r="C62" t="s">
         <v>152</v>
       </c>
     </row>
@@ -1837,9 +2379,9 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1851,7 +2393,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{955EEB82-5C7B-4E05-B07A-7C5BCB435643}">
   <dimension ref="A1:C32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" bestFit="1" customWidth="1"/>
@@ -1937,24 +2479,24 @@
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="14">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="14" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="14">
+      <c r="A9" s="12">
         <v>8</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="14" t="s">
         <v>37</v>
       </c>
     </row>
@@ -2181,7 +2723,251 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:C32" xr:uid="{955EEB82-5C7B-4E05-B07A-7C5BCB435643}"/>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6857A084-77A3-4A97-B947-BCE1F196207E}">
+  <dimension ref="B2:E13"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="2" max="5" width="29.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5">
+      <c r="B2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="B3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C4" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E4" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5">
+      <c r="B7" t="s">
+        <v>160</v>
+      </c>
+      <c r="C7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D7" t="s">
+        <v>160</v>
+      </c>
+      <c r="E7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="B8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C8" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" t="s">
+        <v>161</v>
+      </c>
+      <c r="E8" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5">
+      <c r="B9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C9" t="s">
+        <v>162</v>
+      </c>
+      <c r="D9" t="s">
+        <v>162</v>
+      </c>
+      <c r="E9" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5">
+      <c r="B10" t="s">
+        <v>163</v>
+      </c>
+      <c r="C10" t="s">
+        <v>163</v>
+      </c>
+      <c r="D10" t="s">
+        <v>170</v>
+      </c>
+      <c r="E10" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5">
+      <c r="B11" t="s">
+        <v>164</v>
+      </c>
+      <c r="C11" t="s">
+        <v>164</v>
+      </c>
+      <c r="D11" t="s">
+        <v>164</v>
+      </c>
+      <c r="E11" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5">
+      <c r="B12" t="s">
+        <v>165</v>
+      </c>
+      <c r="C12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D12" t="s">
+        <v>165</v>
+      </c>
+      <c r="E12" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5">
+      <c r="B13" t="s">
+        <v>166</v>
+      </c>
+      <c r="C13" t="s">
+        <v>166</v>
+      </c>
+      <c r="D13" t="s">
+        <v>166</v>
+      </c>
+      <c r="E13" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="B2">
+    <cfRule type="duplicateValues" dxfId="33" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="31"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="duplicateValues" dxfId="30" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="34"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4">
+    <cfRule type="duplicateValues" dxfId="27" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="28"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2">
+    <cfRule type="duplicateValues" dxfId="24" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3">
+    <cfRule type="duplicateValues" dxfId="21" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="22"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4">
+    <cfRule type="duplicateValues" dxfId="18" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2">
+    <cfRule type="duplicateValues" dxfId="14" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2">
+    <cfRule type="duplicateValues" dxfId="13" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3">
+    <cfRule type="duplicateValues" dxfId="10" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4">
+    <cfRule type="duplicateValues" dxfId="8" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2">
+    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2">
+    <cfRule type="duplicateValues" dxfId="5" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E3">
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E4">
+    <cfRule type="duplicateValues" dxfId="1" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="8"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>